<commit_message>
feat(app): advisory report parser + rebalance status engine
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample-advisory.xlsx
+++ b/tests/fixtures/sample-advisory.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I6"/>
+  <dimension ref="A2:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -725,6 +725,25 @@
           <t>No match in holdings</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ESTIMATED TOTAL PROCEEDS — 2 EXITS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>~₹20K</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>